<commit_message>
Preparar el proyecto para multiidioma (español como base)
- Paquete @safetag/i18n: i18next + react-i18next con detección de idioma,
  fallback es, y los términos de dominio comunes (estados, semáforo,
  señales de alarma) que traducen los slugs de la BD.
- Ambas apps inicializan i18n y reemplazan el demo de Vite por un
  placeholder traducido con selector de idioma (oculto mientras solo
  haya uno).
- XLSForm: generador versionado en kobo/gen_xlsform.py con columnas
  label::Idioma (cod); sumar idioma = ampliar LANGS y traducir.
- BD sin cambios: solo guarda slugs estables.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kobo/atc20.xlsx
+++ b/kobo/atc20.xlsx
@@ -431,42 +431,42 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>required</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>appearance</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>hint</t>
+          <t>relevant</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>appearance</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>parameters</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>label::Español (es)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>constraint_message</t>
+          <t>hint::Español (es)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>parameters</t>
+          <t>constraint_message::Español (es)</t>
         </is>
       </c>
     </row>
@@ -543,23 +543,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dirección de la edificación</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Como aparece en la placa, o la más aproximada</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Dirección de la edificación</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Como aparece en la placa, o la más aproximada</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -575,22 +575,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Barrio / comuna</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>${barrio} = 'otro'</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>¿Cuál barrio?</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>${barrio} = 'otro'</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -639,23 +639,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ubicación GPS</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Capturar de pie frente a la edificación, con cielo visible</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ubicación GPS</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Capturar de pie frente a la edificación, con cielo visible</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -671,18 +671,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sistema constructivo</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sistema constructivo</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -699,28 +699,28 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Número de pisos</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 50</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>. &gt;= 1 and . &lt;= 50</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+          <t>Número de pisos</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Debe estar entre 1 y 50</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -735,32 +735,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Señales de alarma observadas</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>not(selected(., 'ninguna') and count-selected(.) &gt; 1)</t>
+          <t>Señales de alarma observadas</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>Marcar todas las que apliquen; si no hay, marcar «Ninguna»</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>«Ninguna» no puede combinarse con otras señales</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -775,28 +775,28 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Foto: fachada completa</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Desde el frente, que se vea todo el edificio</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -811,24 +811,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Foto: esquina 1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Foto: esquina 1</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -843,24 +843,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Foto: esquina 2</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Foto: esquina 2</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -873,22 +873,22 @@
           <t>foto_esquina_3</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Foto: esquina 3 (si es accesible)</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Foto: esquina 3 (si es accesible)</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -901,22 +901,22 @@
           <t>foto_esquina_4</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Foto: esquina 4 (si es accesible)</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Foto: esquina 4 (si es accesible)</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -931,28 +931,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>max-pixels=2048</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Foto: peor grieta, de cerca</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Poner una moneda junto a la grieta como referencia de escala</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>max-pixels=2048</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -967,24 +967,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Foto: columnas del primer piso</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>max-pixels=1600</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Foto: columnas del primer piso</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>max-pixels=1600</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>label::Español (es)</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026081601</t>
+          <t>2026081602</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>